<commit_message>
fix: address Copilot PR review comments
- Fix is_frameshift parsing: explicitly compare string "true" instead of
  bool() which treats "False" as truthy
- Store coverage_fraction as float (12.5, 6.25) instead of truncated int
- Add coverage_label column for unambiguous fraction identification
- Add aggregation column to exp3 metrics to disambiguate overall vs
  per-mutation rows (fixes dupC_ds* naming collision)
- Check BAI existence in completion check, not just BAM
- Seed fallback: parse from filename when provenance.seed is null
- Align non-Docker VNtyper CLI flags (--bam, -o) with actual interface
- Defensive step.get("step") in coverage extraction
- Update classify_sample docstring to accurately describe behavior
- Add is_frameshift assertion to flagged result test
- Update all regex/casting to handle float coverage fractions

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/simulation/tables/supp_table_coverage_titration.xlsx
+++ b/results/simulation/tables/supp_table_coverage_titration.xlsx
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
+        <v>6.25</v>
       </c>
       <c r="C7" t="n">
         <v>100</v>
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="C12" t="n">
         <v>100</v>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>6.25</v>
       </c>
       <c r="C13" t="n">
         <v>100</v>

</xml_diff>